<commit_message>
Add Arabic to language selection, and fix UI for RTL
</commit_message>
<xml_diff>
--- a/documents/Sprint 5/Fliply-Localization.xlsx
+++ b/documents/Sprint 5/Fliply-Localization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ntbngoc/Downloads/Metropolia/Year2/SEP/fliply/documents/Sprint 5/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6E41A715-6541-EC4E-A7F2-40517D3FDE16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B59102FB-7843-7D4F-A093-E2E3EBD1F7CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17480" xr2:uid="{02BBEEC8-28B6-DD4B-8736-C8FDFD175FCF}"/>
+    <workbookView xWindow="-20" yWindow="660" windowWidth="30240" windowHeight="17480" xr2:uid="{02BBEEC8-28B6-DD4B-8736-C8FDFD175FCF}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="912" uniqueCount="639">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1092" uniqueCount="773">
   <si>
     <t>Key</t>
   </si>
@@ -1963,6 +1963,408 @@
   </si>
   <si>
     <t>Trắc nghiệm</t>
+  </si>
+  <si>
+    <t>AR</t>
+  </si>
+  <si>
+    <t>اللغة</t>
+  </si>
+  <si>
+    <t>تعلم سريع وسهل</t>
+  </si>
+  <si>
+    <t>التسجيل</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> تسجيل الدخول</t>
+  </si>
+  <si>
+    <t>أدخل بيانات تسجيل الدخول الخاصة بك للوصول إلى حسابك</t>
+  </si>
+  <si>
+    <t>بريد إلكتروني</t>
+  </si>
+  <si>
+    <t>كلمة المرور</t>
+  </si>
+  <si>
+    <t>هل نسيت كلمة المرور؟</t>
+  </si>
+  <si>
+    <t>تسجيل الدخول</t>
+  </si>
+  <si>
+    <t>ليس لديك حساب؟</t>
+  </si>
+  <si>
+    <t>اشتراك</t>
+  </si>
+  <si>
+    <t>بريد إلكتروني أو كلمة مرور غير صحيحة</t>
+  </si>
+  <si>
+    <t>يسجل</t>
+  </si>
+  <si>
+    <t>إنشاء حساب</t>
+  </si>
+  <si>
+    <t>الاسم الأول</t>
+  </si>
+  <si>
+    <t>اسم العائلة</t>
+  </si>
+  <si>
+    <t>هل أنت معلم؟</t>
+  </si>
+  <si>
+    <t>نعم</t>
+  </si>
+  <si>
+    <t>لا</t>
+  </si>
+  <si>
+    <t>بإنشاء حساب، فإنك توافق على الشروط والأحكام الخاصة بنا.</t>
+  </si>
+  <si>
+    <t>هل لديك حساب بالفعل؟</t>
+  </si>
+  <si>
+    <t>يرجى الموافقة على الشروط والأحكام.</t>
+  </si>
+  <si>
+    <t>يرجى ملء جميع الحقول.</t>
+  </si>
+  <si>
+    <t>register.warning.invalidEmail</t>
+  </si>
+  <si>
+    <t>البريد الإلكتروني غير صالح.</t>
+  </si>
+  <si>
+    <t>register.warning.passwordTooShort</t>
+  </si>
+  <si>
+    <t>يجب أن تتكون كلمة المرور من 6 أحرف على الأقل.</t>
+  </si>
+  <si>
+    <t>register.warning.emailExists</t>
+  </si>
+  <si>
+    <t>البريد الإلكتروني موجود بالفعل.</t>
+  </si>
+  <si>
+    <t>register.warning.dbError</t>
+  </si>
+  <si>
+    <t>فشل التسجيل (خطأ في قاعدة البيانات).</t>
+  </si>
+  <si>
+    <t>Email is not valid.</t>
+  </si>
+  <si>
+    <t>Password must be at least 6 characters.</t>
+  </si>
+  <si>
+    <t>Email already exists.</t>
+  </si>
+  <si>
+    <t>Register failed (database error).</t>
+  </si>
+  <si>
+    <t>Sähköposti ei ole kelvollinen.</t>
+  </si>
+  <si>
+    <t>Salasanassa on oltava vähintään 6 merkkiä.</t>
+  </si>
+  <si>
+    <t>Sähköposti on jo olemassa.</t>
+  </si>
+  <si>
+    <t>Rekisteröityminen epäonnistui (tietokantavirhe).</t>
+  </si>
+  <si>
+    <t>유효하지 않은 이메일입니다.</t>
+  </si>
+  <si>
+    <t>비밀번호는 최소 6자 이상이어야 합니다.</t>
+  </si>
+  <si>
+    <t>이미 존재하는 이메일입니다.</t>
+  </si>
+  <si>
+    <t>회원가입에 실패했습니다(데이터베이스 오류).</t>
+  </si>
+  <si>
+    <t>ອີເມວບໍ່ຖືກຕ້ອງ.</t>
+  </si>
+  <si>
+    <t>ລະຫັດຜ່ານຕ້ອງຍາວຢ່າງໜ້ອຍ 6 ຕົວອັກສອນ.</t>
+  </si>
+  <si>
+    <t>ອີເມວນີ້ມີຢູ່ແລ້ວ.</t>
+  </si>
+  <si>
+    <t>ລົງທະບຽນບໍ່ສໍາເລັດ (ຜິດພາດຖານຂໍ້ມູນ).</t>
+  </si>
+  <si>
+    <t>Email không hợp lệ.</t>
+  </si>
+  <si>
+    <t>Mật khẩu phải có ít nhất 6 ký tự.</t>
+  </si>
+  <si>
+    <t>Email đã tồn tại.</t>
+  </si>
+  <si>
+    <t>Đăng ký thất bại (lỗi cơ sở dữ liệu).</t>
+  </si>
+  <si>
+    <t>بيت</t>
+  </si>
+  <si>
+    <t>فصول</t>
+  </si>
+  <si>
+    <t>البطاقات التعليمية</t>
+  </si>
+  <si>
+    <t>مسابقات</t>
+  </si>
+  <si>
+    <t>حساب</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> تحرير الحساب</t>
+  </si>
+  <si>
+    <t>تغيير كلمة المرور</t>
+  </si>
+  <si>
+    <t>يساعد</t>
+  </si>
+  <si>
+    <t>معلومات عنا</t>
+  </si>
+  <si>
+    <t>تسجيل الخروج</t>
+  </si>
+  <si>
+    <t>يحرر</t>
+  </si>
+  <si>
+    <t>يمسح</t>
+  </si>
+  <si>
+    <t>حسابي</t>
+  </si>
+  <si>
+    <t>المستخدم غير مسجل الدخول.</t>
+  </si>
+  <si>
+    <t>كلمة المرور الحالية غير صحيحة.</t>
+  </si>
+  <si>
+    <t>يجب أن تتكون كلمة المرور الجديدة من 6 أحرف على الأقل.</t>
+  </si>
+  <si>
+    <t>كلمة المرور الجديدة وكلمة المرور المؤكدة لا تتطابقان.</t>
+  </si>
+  <si>
+    <t>Fliply هو تطبيق تعليمي إلكتروني يعتمد على البطاقات التعليمية، مصمم خصيصًا للطلاب والمعلمين على حد سواء. يوفر التطبيق طريقة سهلة وفعّالة لإنشاء وتنظيم ودراسة المواد التعليمية في مكان واحد. سواء كنت تستعد للامتحانات، أو تُدرّس فصلًا دراسيًا، أو تتعلم شيئًا جديدًا، فإن Fliply مصمم لجعل الدراسة أكثر متعة وكفاءة.</t>
+  </si>
+  <si>
+    <t>يحفظ</t>
+  </si>
+  <si>
+    <t>يلغي</t>
+  </si>
+  <si>
+    <t>كيفية استخدام هذا التطبيق…</t>
+  </si>
+  <si>
+    <t>كلمة المرور الحالية</t>
+  </si>
+  <si>
+    <t>كلمة المرور الجديدة</t>
+  </si>
+  <si>
+    <t>تأكيد كلمة المرور الجديدة</t>
+  </si>
+  <si>
+    <t>عنوان</t>
+  </si>
+  <si>
+    <t>الترجمة</t>
+  </si>
+  <si>
+    <t>أهلاً،</t>
+  </si>
+  <si>
+    <t>لنبدأ التعلم</t>
+  </si>
+  <si>
+    <t>أحدث فئة</t>
+  </si>
+  <si>
+    <t>أحدث مسابقة</t>
+  </si>
+  <si>
+    <t>إدارة الفصول الدراسية الخاصة بك</t>
+  </si>
+  <si>
+    <t>تعذر تحميل الصفحة</t>
+  </si>
+  <si>
+    <t>صفي</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> الفصول الدراسية الخاصة بك المسجلين</t>
+  </si>
+  <si>
+    <t>فشل تحميل ملف class_card.fxml</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> إضافة المزيد من الفصول+</t>
+  </si>
+  <si>
+    <t>مسابقة جديدة</t>
+  </si>
+  <si>
+    <t>رمز الفصل</t>
+  </si>
+  <si>
+    <t>يضيف</t>
+  </si>
+  <si>
+    <t>فئة جديدة</t>
+  </si>
+  <si>
+    <t>خطأ</t>
+  </si>
+  <si>
+    <t>مدرس</t>
+  </si>
+  <si>
+    <t>طلاب</t>
+  </si>
+  <si>
+    <t>إضافة المزيد من الطلاب+</t>
+  </si>
+  <si>
+    <t>بحث الطالب…</t>
+  </si>
+  <si>
+    <t>يغلق</t>
+  </si>
+  <si>
+    <t>مجموعات البطاقات التعليمية</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> أضف المزيد من مجموعات البطاقات التعليمية+</t>
+  </si>
+  <si>
+    <t>لا توجد بطاقات تعليمية متاحة (أو رقم غير صالح).</t>
+  </si>
+  <si>
+    <t>عدد الأسئلة</t>
+  </si>
+  <si>
+    <t>أدخل عدد الأسئلة</t>
+  </si>
+  <si>
+    <t>يولد</t>
+  </si>
+  <si>
+    <t>اختبار #{0}</t>
+  </si>
+  <si>
+    <t>مجموع النقاط: {0}</t>
+  </si>
+  <si>
+    <t>عرض النتيجة</t>
+  </si>
+  <si>
+    <t>اختباراتي</t>
+  </si>
+  <si>
+    <t>المجموع: {0}</t>
+  </si>
+  <si>
+    <t>نتيجة</t>
+  </si>
+  <si>
+    <t>صحيح</t>
+  </si>
+  <si>
+    <t>غير صحيح</t>
+  </si>
+  <si>
+    <t>لم يتم الرد</t>
+  </si>
+  <si>
+    <t>أعد تشغيل الاختبار</t>
+  </si>
+  <si>
+    <t>العودة إلى الاختبارات</t>
+  </si>
+  <si>
+    <t>مجموعة جديدة من البطاقات التعليمية</t>
+  </si>
+  <si>
+    <t>موضوع</t>
+  </si>
+  <si>
+    <t>تحميل الملف</t>
+  </si>
+  <si>
+    <t>تم تحميل: {0} ({1} بطاقة)</t>
+  </si>
+  <si>
+    <t>لا يمكن قراءة الملف.</t>
+  </si>
+  <si>
+    <t>لمجموع: {0}</t>
+  </si>
+  <si>
+    <t>شرط</t>
+  </si>
+  <si>
+    <t>تعريف</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> أضف المزيد من البطاقات التعليمية+</t>
+  </si>
+  <si>
+    <t>البطاقات التعليمية الخاصة بي</t>
+  </si>
+  <si>
+    <t>المجموع:</t>
+  </si>
+  <si>
+    <t>فشل تحميل ملف term_tile.fxml</t>
+  </si>
+  <si>
+    <t>تحرير البطاقات التعليمية</t>
+  </si>
+  <si>
+    <t>بطاقة تعليمية جديدة</t>
+  </si>
+  <si>
+    <t>Total:</t>
+  </si>
+  <si>
+    <t>Yhteensä:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">총 개수: </t>
+  </si>
+  <si>
+    <t>ທັງໝົດ:</t>
+  </si>
+  <si>
+    <t>Tổng:</t>
   </si>
 </sst>
 </file>
@@ -2129,7 +2531,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2156,6 +2558,8 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2490,18 +2894,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A16CBA21-4DE3-6C40-8146-BCE7D2C09174}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.6640625" customWidth="1"/>
-    <col min="2" max="2" width="28.5" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="31.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="35.1640625" customWidth="1"/>
+    <col min="2" max="3" width="28.5" customWidth="1"/>
+    <col min="4" max="4" width="30.83203125" customWidth="1"/>
+    <col min="5" max="5" width="31.83203125" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="35.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2509,19 +2913,22 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>639</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -2529,19 +2936,22 @@
         <v>7</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>640</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -2560,8 +2970,11 @@
       <c r="F3" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G3" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -2569,19 +2982,22 @@
         <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>641</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
@@ -2589,19 +3005,22 @@
         <v>20</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>642</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>25</v>
       </c>
@@ -2609,15 +3028,18 @@
         <v>26</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>643</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2628,18 +3050,19 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA477C81-485F-A245-9AA1-F07915094CCD}">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.5" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="31.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="35.1640625" customWidth="1"/>
+    <col min="3" max="3" width="27.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.83203125" customWidth="1"/>
+    <col min="5" max="5" width="31.83203125" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="35.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2647,19 +3070,22 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>639</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>383</v>
       </c>
@@ -2667,19 +3093,22 @@
         <v>384</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>754</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>385</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>387</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>389</v>
       </c>
@@ -2687,19 +3116,22 @@
         <v>390</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>755</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>395</v>
       </c>
@@ -2707,19 +3139,22 @@
         <v>396</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>756</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>397</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>400</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>401</v>
       </c>
@@ -2727,19 +3162,22 @@
         <v>402</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>757</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>404</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>405</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>406</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>407</v>
       </c>
@@ -2747,19 +3185,22 @@
         <v>408</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>758</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>409</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>410</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>411</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>412</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>413</v>
       </c>
@@ -2767,19 +3208,22 @@
         <v>297</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>729</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>299</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>415</v>
       </c>
@@ -2787,19 +3231,22 @@
         <v>176</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>710</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>416</v>
       </c>
@@ -2807,19 +3254,22 @@
         <v>417</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>759</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>421</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>422</v>
       </c>
@@ -2827,19 +3277,22 @@
         <v>423</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>760</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>424</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>425</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>426</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>428</v>
       </c>
@@ -2847,19 +3300,22 @@
         <v>429</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>761</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="E11" s="1" t="s">
         <v>431</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="F11" s="1" t="s">
         <v>432</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>433</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>434</v>
       </c>
@@ -2867,19 +3323,22 @@
         <v>170</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>709</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>435</v>
       </c>
@@ -2887,19 +3346,22 @@
         <v>176</v>
       </c>
       <c r="C13" s="1" t="s">
+        <v>710</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="E13" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>436</v>
       </c>
@@ -2907,15 +3369,18 @@
         <v>437</v>
       </c>
       <c r="C14" s="12" t="s">
+        <v>762</v>
+      </c>
+      <c r="D14" s="12" t="s">
         <v>438</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="E14" s="1" t="s">
         <v>439</v>
       </c>
-      <c r="E14" s="12" t="s">
+      <c r="F14" s="12" t="s">
         <v>440</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>441</v>
       </c>
     </row>
@@ -2926,38 +3391,42 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15BD5F0E-16B6-A147-812F-6ADFED0BEF74}">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.1640625" style="6" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36.1640625" style="13" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="45.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="65" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="52" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.1640625" style="13" customWidth="1"/>
+    <col min="4" max="4" width="45.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="65" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="35.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="52" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="16" t="s">
+        <v>639</v>
+      </c>
+      <c r="D1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="E1" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="F1" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="G1" s="15" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="14" t="s">
         <v>442</v>
       </c>
@@ -2965,19 +3434,22 @@
         <v>443</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>727</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>444</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>445</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>446</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>447</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="14" t="s">
         <v>448</v>
       </c>
@@ -2985,19 +3457,22 @@
         <v>449</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>739</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>450</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>453</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="14" t="s">
         <v>454</v>
       </c>
@@ -3005,19 +3480,22 @@
         <v>455</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>740</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>457</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>458</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>459</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="14" t="s">
         <v>460</v>
       </c>
@@ -3025,19 +3503,22 @@
         <v>461</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>741</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>462</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>463</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>465</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
         <v>466</v>
       </c>
@@ -3045,19 +3526,22 @@
         <v>467</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>742</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>468</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>469</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>470</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>471</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="14" t="s">
         <v>472</v>
       </c>
@@ -3065,19 +3549,22 @@
         <v>176</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>710</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="14" t="s">
         <v>473</v>
       </c>
@@ -3085,19 +3572,22 @@
         <v>474</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>475</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>476</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>477</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>478</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="14" t="s">
         <v>479</v>
       </c>
@@ -3105,19 +3595,22 @@
         <v>480</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>744</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>481</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>482</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>483</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>484</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="14" t="s">
         <v>485</v>
       </c>
@@ -3125,19 +3618,22 @@
         <v>486</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>745</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>487</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>489</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>490</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="14" t="s">
         <v>491</v>
       </c>
@@ -3145,19 +3641,22 @@
         <v>492</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>746</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="E11" s="1" t="s">
         <v>494</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="F11" s="1" t="s">
         <v>495</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>496</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="14" t="s">
         <v>497</v>
       </c>
@@ -3165,19 +3664,22 @@
         <v>417</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>747</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>498</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="14" t="s">
         <v>499</v>
       </c>
@@ -3185,19 +3687,22 @@
         <v>500</v>
       </c>
       <c r="C13" s="1" t="s">
+        <v>748</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>501</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="E13" s="1" t="s">
         <v>502</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>503</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>504</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="14" t="s">
         <v>505</v>
       </c>
@@ -3205,19 +3710,22 @@
         <v>480</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>744</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>481</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="E14" s="1" t="s">
         <v>482</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="F14" s="1" t="s">
         <v>483</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>484</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="14" t="s">
         <v>506</v>
       </c>
@@ -3225,19 +3733,22 @@
         <v>507</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>749</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>508</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="E15" s="1" t="s">
         <v>509</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="F15" s="1" t="s">
         <v>510</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>511</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="14" t="s">
         <v>512</v>
       </c>
@@ -3245,19 +3756,22 @@
         <v>513</v>
       </c>
       <c r="C16" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>514</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="E16" s="1" t="s">
         <v>515</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>516</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>517</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="14" t="s">
         <v>518</v>
       </c>
@@ -3265,19 +3779,22 @@
         <v>519</v>
       </c>
       <c r="C17" s="1" t="s">
+        <v>751</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>520</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="E17" s="1" t="s">
         <v>521</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="F17" s="1" t="s">
         <v>522</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="1" t="s">
         <v>523</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="14" t="s">
         <v>524</v>
       </c>
@@ -3285,19 +3802,22 @@
         <v>525</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>752</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>526</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="E18" s="1" t="s">
         <v>527</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="F18" s="1" t="s">
         <v>528</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>529</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="14" t="s">
         <v>530</v>
       </c>
@@ -3305,15 +3825,18 @@
         <v>531</v>
       </c>
       <c r="C19" s="1" t="s">
+        <v>753</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>532</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="E19" s="1" t="s">
         <v>533</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="F19" s="1" t="s">
         <v>534</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="G19" s="1" t="s">
         <v>535</v>
       </c>
     </row>
@@ -3324,18 +3847,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0392508-4C52-9446-AA8D-271D6068BC34}">
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.6640625" customWidth="1"/>
     <col min="2" max="2" width="39" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="41.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="30.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39" customWidth="1"/>
+    <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="41.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -3343,19 +3867,22 @@
         <v>1</v>
       </c>
       <c r="C1" s="8" t="s">
+        <v>639</v>
+      </c>
+      <c r="D1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="E1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="F1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="G1" s="8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="22" t="s">
         <v>31</v>
       </c>
@@ -3363,19 +3890,22 @@
         <v>32</v>
       </c>
       <c r="C2" s="9" t="s">
+        <v>643</v>
+      </c>
+      <c r="D2" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="E2" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="F2" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="G2" s="9" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="22" t="s">
         <v>34</v>
       </c>
@@ -3383,19 +3913,22 @@
         <v>35</v>
       </c>
       <c r="C3" s="9" t="s">
+        <v>644</v>
+      </c>
+      <c r="D3" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="E3" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="F3" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="G3" s="9" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="22" t="s">
         <v>40</v>
       </c>
@@ -3403,19 +3936,22 @@
         <v>41</v>
       </c>
       <c r="C4" s="9" t="s">
+        <v>645</v>
+      </c>
+      <c r="D4" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="E4" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="F4" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="22" t="s">
         <v>45</v>
       </c>
@@ -3423,19 +3959,22 @@
         <v>46</v>
       </c>
       <c r="C5" s="9" t="s">
+        <v>646</v>
+      </c>
+      <c r="D5" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="E5" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="F5" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="G5" s="9" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="22" t="s">
         <v>51</v>
       </c>
@@ -3443,19 +3982,22 @@
         <v>41</v>
       </c>
       <c r="C6" s="9" t="s">
+        <v>645</v>
+      </c>
+      <c r="D6" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="E6" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="F6" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="G6" s="9" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="22" t="s">
         <v>52</v>
       </c>
@@ -3463,19 +4005,22 @@
         <v>46</v>
       </c>
       <c r="C7" s="9" t="s">
+        <v>646</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="E7" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="F7" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="G7" s="9" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="22" t="s">
         <v>53</v>
       </c>
@@ -3483,19 +4028,22 @@
         <v>54</v>
       </c>
       <c r="C8" s="9" t="s">
+        <v>647</v>
+      </c>
+      <c r="D8" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="E8" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="F8" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="G8" s="9" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="22" t="s">
         <v>59</v>
       </c>
@@ -3503,19 +4051,22 @@
         <v>32</v>
       </c>
       <c r="C9" s="9" t="s">
+        <v>648</v>
+      </c>
+      <c r="D9" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="E9" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="F9" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="G9" s="9" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="22" t="s">
         <v>61</v>
       </c>
@@ -3523,19 +4074,22 @@
         <v>62</v>
       </c>
       <c r="C10" s="9" t="s">
+        <v>649</v>
+      </c>
+      <c r="D10" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="E10" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="F10" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="G10" s="9" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="22" t="s">
         <v>67</v>
       </c>
@@ -3543,19 +4097,22 @@
         <v>68</v>
       </c>
       <c r="C11" s="9" t="s">
+        <v>650</v>
+      </c>
+      <c r="D11" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="E11" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="F11" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="G11" s="9" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="22" t="s">
         <v>69</v>
       </c>
@@ -3563,25 +4120,29 @@
         <v>70</v>
       </c>
       <c r="C12" s="9" t="s">
+        <v>651</v>
+      </c>
+      <c r="D12" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="E12" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="F12" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="G12" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="6"/>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
       <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
     </row>
     <row r="26" spans="1:1" ht="32" x14ac:dyDescent="0.4">
       <c r="A26" s="5"/>
@@ -3656,18 +4217,19 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F107B45-44C2-6E4C-B453-9E61ED0D571C}">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="47.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="33.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="56.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.5" customWidth="1"/>
+    <col min="4" max="4" width="32.33203125" customWidth="1"/>
+    <col min="5" max="5" width="37" customWidth="1"/>
+    <col min="6" max="6" width="33.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="56.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -3675,19 +4237,22 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>639</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="23" t="s">
         <v>567</v>
       </c>
@@ -3695,19 +4260,22 @@
         <v>20</v>
       </c>
       <c r="C2" s="21" t="s">
+        <v>652</v>
+      </c>
+      <c r="D2" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="E2" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="F2" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="G2" s="21" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="23" t="s">
         <v>568</v>
       </c>
@@ -3715,19 +4283,22 @@
         <v>569</v>
       </c>
       <c r="C3" s="21" t="s">
+        <v>653</v>
+      </c>
+      <c r="D3" s="21" t="s">
         <v>570</v>
       </c>
-      <c r="D3" s="21" t="s">
+      <c r="E3" s="21" t="s">
         <v>571</v>
       </c>
-      <c r="E3" s="21" t="s">
+      <c r="F3" s="21" t="s">
         <v>572</v>
       </c>
-      <c r="F3" s="21" t="s">
+      <c r="G3" s="21" t="s">
         <v>573</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="23" t="s">
         <v>574</v>
       </c>
@@ -3735,19 +4306,22 @@
         <v>157</v>
       </c>
       <c r="C4" s="21" t="s">
+        <v>654</v>
+      </c>
+      <c r="D4" s="21" t="s">
         <v>158</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="E4" s="21" t="s">
         <v>159</v>
       </c>
-      <c r="E4" s="21" t="s">
+      <c r="F4" s="21" t="s">
         <v>160</v>
       </c>
-      <c r="F4" s="21" t="s">
+      <c r="G4" s="21" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="23" t="s">
         <v>575</v>
       </c>
@@ -3755,19 +4329,22 @@
         <v>157</v>
       </c>
       <c r="C5" s="21" t="s">
+        <v>654</v>
+      </c>
+      <c r="D5" s="21" t="s">
         <v>158</v>
       </c>
-      <c r="D5" s="21" t="s">
+      <c r="E5" s="21" t="s">
         <v>159</v>
       </c>
-      <c r="E5" s="21" t="s">
+      <c r="F5" s="21" t="s">
         <v>160</v>
       </c>
-      <c r="F5" s="21" t="s">
+      <c r="G5" s="21" t="s">
         <v>576</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="23" t="s">
         <v>577</v>
       </c>
@@ -3775,19 +4352,22 @@
         <v>163</v>
       </c>
       <c r="C6" s="21" t="s">
+        <v>655</v>
+      </c>
+      <c r="D6" s="21" t="s">
         <v>164</v>
       </c>
-      <c r="D6" s="21" t="s">
+      <c r="E6" s="21" t="s">
         <v>165</v>
       </c>
-      <c r="E6" s="21" t="s">
+      <c r="F6" s="21" t="s">
         <v>166</v>
       </c>
-      <c r="F6" s="21" t="s">
+      <c r="G6" s="21" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="23" t="s">
         <v>578</v>
       </c>
@@ -3795,19 +4375,22 @@
         <v>163</v>
       </c>
       <c r="C7" s="21" t="s">
+        <v>655</v>
+      </c>
+      <c r="D7" s="21" t="s">
         <v>164</v>
       </c>
-      <c r="D7" s="21" t="s">
+      <c r="E7" s="21" t="s">
         <v>165</v>
       </c>
-      <c r="E7" s="21" t="s">
+      <c r="F7" s="21" t="s">
         <v>166</v>
       </c>
-      <c r="F7" s="21" t="s">
+      <c r="G7" s="21" t="s">
         <v>579</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="23" t="s">
         <v>580</v>
       </c>
@@ -3815,19 +4398,22 @@
         <v>41</v>
       </c>
       <c r="C8" s="21" t="s">
+        <v>645</v>
+      </c>
+      <c r="D8" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="E8" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="E8" s="21" t="s">
+      <c r="F8" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="F8" s="21" t="s">
+      <c r="G8" s="21" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="23" t="s">
         <v>581</v>
       </c>
@@ -3835,19 +4421,22 @@
         <v>41</v>
       </c>
       <c r="C9" s="21" t="s">
+        <v>645</v>
+      </c>
+      <c r="D9" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="21" t="s">
+      <c r="E9" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="21" t="s">
+      <c r="F9" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="F9" s="21" t="s">
+      <c r="G9" s="21" t="s">
         <v>582</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="23" t="s">
         <v>583</v>
       </c>
@@ -3855,19 +4444,22 @@
         <v>46</v>
       </c>
       <c r="C10" s="21" t="s">
+        <v>646</v>
+      </c>
+      <c r="D10" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="21" t="s">
+      <c r="E10" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="21" t="s">
+      <c r="F10" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="F10" s="21" t="s">
+      <c r="G10" s="21" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="23" t="s">
         <v>584</v>
       </c>
@@ -3875,19 +4467,22 @@
         <v>46</v>
       </c>
       <c r="C11" s="21" t="s">
+        <v>646</v>
+      </c>
+      <c r="D11" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="21" t="s">
+      <c r="E11" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="21" t="s">
+      <c r="F11" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="F11" s="21" t="s">
+      <c r="G11" s="21" t="s">
         <v>585</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="23" t="s">
         <v>586</v>
       </c>
@@ -3895,19 +4490,22 @@
         <v>587</v>
       </c>
       <c r="C12" s="21" t="s">
+        <v>656</v>
+      </c>
+      <c r="D12" s="21" t="s">
         <v>588</v>
       </c>
-      <c r="D12" s="21" t="s">
+      <c r="E12" s="21" t="s">
         <v>589</v>
       </c>
-      <c r="E12" s="21" t="s">
+      <c r="F12" s="21" t="s">
         <v>590</v>
       </c>
-      <c r="F12" s="21" t="s">
+      <c r="G12" s="21" t="s">
         <v>591</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="23" t="s">
         <v>592</v>
       </c>
@@ -3915,19 +4513,22 @@
         <v>593</v>
       </c>
       <c r="C13" s="21" t="s">
+        <v>657</v>
+      </c>
+      <c r="D13" s="21" t="s">
         <v>594</v>
       </c>
-      <c r="D13" s="21" t="s">
+      <c r="E13" s="21" t="s">
         <v>595</v>
       </c>
-      <c r="E13" s="21" t="s">
+      <c r="F13" s="21" t="s">
         <v>596</v>
       </c>
-      <c r="F13" s="21" t="s">
+      <c r="G13" s="21" t="s">
         <v>597</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="23" t="s">
         <v>598</v>
       </c>
@@ -3935,19 +4536,22 @@
         <v>599</v>
       </c>
       <c r="C14" s="21" t="s">
+        <v>658</v>
+      </c>
+      <c r="D14" s="21" t="s">
         <v>600</v>
       </c>
-      <c r="D14" s="21" t="s">
+      <c r="E14" s="21" t="s">
         <v>601</v>
       </c>
-      <c r="E14" s="21" t="s">
+      <c r="F14" s="21" t="s">
         <v>602</v>
       </c>
-      <c r="F14" s="21" t="s">
+      <c r="G14" s="21" t="s">
         <v>603</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="23" t="s">
         <v>604</v>
       </c>
@@ -3955,19 +4559,22 @@
         <v>605</v>
       </c>
       <c r="C15" s="21" t="s">
+        <v>659</v>
+      </c>
+      <c r="D15" s="21" t="s">
         <v>606</v>
       </c>
-      <c r="D15" s="21" t="s">
+      <c r="E15" s="21" t="s">
         <v>607</v>
       </c>
-      <c r="E15" s="21" t="s">
+      <c r="F15" s="21" t="s">
         <v>608</v>
       </c>
-      <c r="F15" s="21" t="s">
+      <c r="G15" s="21" t="s">
         <v>609</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="23" t="s">
         <v>610</v>
       </c>
@@ -3975,19 +4582,22 @@
         <v>20</v>
       </c>
       <c r="C16" s="21" t="s">
+        <v>652</v>
+      </c>
+      <c r="D16" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="D16" s="21" t="s">
+      <c r="E16" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="E16" s="21" t="s">
+      <c r="F16" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="F16" s="21" t="s">
+      <c r="G16" s="21" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="23" t="s">
         <v>611</v>
       </c>
@@ -3995,19 +4605,22 @@
         <v>612</v>
       </c>
       <c r="C17" s="21" t="s">
+        <v>660</v>
+      </c>
+      <c r="D17" s="21" t="s">
         <v>613</v>
       </c>
-      <c r="D17" s="21" t="s">
+      <c r="E17" s="21" t="s">
         <v>614</v>
       </c>
-      <c r="E17" s="21" t="s">
+      <c r="F17" s="21" t="s">
         <v>615</v>
       </c>
-      <c r="F17" s="21" t="s">
+      <c r="G17" s="21" t="s">
         <v>616</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="23" t="s">
         <v>617</v>
       </c>
@@ -4015,19 +4628,22 @@
         <v>618</v>
       </c>
       <c r="C18" s="21" t="s">
+        <v>648</v>
+      </c>
+      <c r="D18" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="D18" s="21" t="s">
+      <c r="E18" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="E18" s="21" t="s">
+      <c r="F18" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="F18" s="21" t="s">
+      <c r="G18" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="23" t="s">
         <v>619</v>
       </c>
@@ -4035,19 +4651,22 @@
         <v>20</v>
       </c>
       <c r="C19" s="21" t="s">
+        <v>652</v>
+      </c>
+      <c r="D19" s="21" t="s">
         <v>620</v>
       </c>
-      <c r="D19" s="21" t="s">
+      <c r="E19" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="E19" s="21" t="s">
+      <c r="F19" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="F19" s="21" t="s">
+      <c r="G19" s="21" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="23" t="s">
         <v>621</v>
       </c>
@@ -4055,19 +4674,22 @@
         <v>622</v>
       </c>
       <c r="C20" s="21" t="s">
+        <v>661</v>
+      </c>
+      <c r="D20" s="21" t="s">
         <v>623</v>
       </c>
-      <c r="D20" s="21" t="s">
+      <c r="E20" s="21" t="s">
         <v>624</v>
       </c>
-      <c r="E20" s="21" t="s">
+      <c r="F20" s="21" t="s">
         <v>625</v>
       </c>
-      <c r="F20" s="21" t="s">
+      <c r="G20" s="21" t="s">
         <v>626</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="23" t="s">
         <v>627</v>
       </c>
@@ -4075,29 +4697,125 @@
         <v>628</v>
       </c>
       <c r="C21" s="21" t="s">
+        <v>662</v>
+      </c>
+      <c r="D21" s="21" t="s">
         <v>629</v>
       </c>
-      <c r="D21" s="21" t="s">
+      <c r="E21" s="21" t="s">
         <v>630</v>
       </c>
-      <c r="E21" s="21" t="s">
+      <c r="F21" s="21" t="s">
         <v>631</v>
       </c>
-      <c r="F21" s="21" t="s">
+      <c r="G21" s="21" t="s">
         <v>632</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" s="24" t="s">
+        <v>663</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>671</v>
+      </c>
+      <c r="C22" s="25" t="s">
+        <v>664</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>675</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>679</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>683</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" s="24" t="s">
+        <v>665</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>672</v>
+      </c>
+      <c r="C23" s="25" t="s">
+        <v>666</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>676</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>680</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>684</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24" s="24" t="s">
+        <v>667</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>673</v>
+      </c>
+      <c r="C24" s="25" t="s">
+        <v>668</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>677</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>681</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>685</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" s="24" t="s">
+        <v>669</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>674</v>
+      </c>
+      <c r="C25" s="25" t="s">
+        <v>670</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>678</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>682</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>690</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E59BFD5-A707-4B36-9E6D-F9516EA5BE28}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="15.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -4105,19 +4823,22 @@
         <v>1</v>
       </c>
       <c r="C1" s="8" t="s">
+        <v>639</v>
+      </c>
+      <c r="D1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="E1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="F1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="G1" s="8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="22" t="s">
         <v>226</v>
       </c>
@@ -4125,19 +4846,22 @@
         <v>227</v>
       </c>
       <c r="C2" s="9" t="s">
+        <v>691</v>
+      </c>
+      <c r="D2" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="E2" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="F2" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="G2" s="9" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="22" t="s">
         <v>232</v>
       </c>
@@ -4145,19 +4869,22 @@
         <v>233</v>
       </c>
       <c r="C3" s="9" t="s">
+        <v>692</v>
+      </c>
+      <c r="D3" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="E3" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="F3" s="9" t="s">
         <v>236</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="G3" s="9" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="22" t="s">
         <v>238</v>
       </c>
@@ -4165,19 +4892,22 @@
         <v>239</v>
       </c>
       <c r="C4" s="9" t="s">
+        <v>693</v>
+      </c>
+      <c r="D4" s="9" t="s">
         <v>240</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="E4" s="9" t="s">
         <v>241</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="F4" s="9" t="s">
         <v>242</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="22" t="s">
         <v>244</v>
       </c>
@@ -4185,19 +4915,22 @@
         <v>245</v>
       </c>
       <c r="C5" s="9" t="s">
+        <v>694</v>
+      </c>
+      <c r="D5" s="9" t="s">
         <v>246</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="E5" s="9" t="s">
         <v>247</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="F5" s="9" t="s">
         <v>248</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="G5" s="9" t="s">
         <v>638</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="22" t="s">
         <v>249</v>
       </c>
@@ -4205,15 +4938,18 @@
         <v>250</v>
       </c>
       <c r="C6" s="9" t="s">
+        <v>695</v>
+      </c>
+      <c r="D6" s="9" t="s">
         <v>251</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="E6" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="F6" s="9" t="s">
         <v>253</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="G6" s="9" t="s">
         <v>254</v>
       </c>
     </row>
@@ -4224,18 +4960,18 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BBF0CD9-760D-164D-962F-465690924422}">
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="45.1640625" customWidth="1"/>
-    <col min="3" max="3" width="41.5" customWidth="1"/>
-    <col min="4" max="4" width="47.5" customWidth="1"/>
-    <col min="5" max="5" width="41" customWidth="1"/>
-    <col min="6" max="6" width="41.33203125" customWidth="1"/>
+    <col min="2" max="3" width="45.1640625" customWidth="1"/>
+    <col min="4" max="4" width="41.5" customWidth="1"/>
+    <col min="5" max="5" width="47.5" customWidth="1"/>
+    <col min="6" max="6" width="41" customWidth="1"/>
+    <col min="7" max="7" width="41.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -4243,19 +4979,22 @@
         <v>1</v>
       </c>
       <c r="C1" s="10" t="s">
+        <v>639</v>
+      </c>
+      <c r="D1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="E1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="F1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="G1" s="10" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>75</v>
       </c>
@@ -4263,19 +5002,22 @@
         <v>76</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>81</v>
       </c>
@@ -4283,19 +5025,22 @@
         <v>82</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>697</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>87</v>
       </c>
@@ -4303,19 +5048,22 @@
         <v>88</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>93</v>
       </c>
@@ -4323,19 +5071,22 @@
         <v>94</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>699</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>99</v>
       </c>
@@ -4343,19 +5094,22 @@
         <v>100</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>700</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>105</v>
       </c>
@@ -4363,19 +5117,22 @@
         <v>106</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>701</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>111</v>
       </c>
@@ -4383,19 +5140,22 @@
         <v>112</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>702</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>117</v>
       </c>
@@ -4403,19 +5163,22 @@
         <v>118</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>703</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>123</v>
       </c>
@@ -4423,19 +5186,22 @@
         <v>124</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>699</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>125</v>
       </c>
@@ -4443,19 +5209,22 @@
         <v>126</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="E11" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="F11" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>127</v>
       </c>
@@ -4463,19 +5232,22 @@
         <v>88</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>128</v>
       </c>
@@ -4483,19 +5255,22 @@
         <v>129</v>
       </c>
       <c r="C13" s="1" t="s">
+        <v>697</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="E13" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>130</v>
       </c>
@@ -4503,19 +5278,22 @@
         <v>131</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>704</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="E14" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="F14" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>136</v>
       </c>
@@ -4523,19 +5301,22 @@
         <v>137</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>705</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="E15" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="F15" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>142</v>
       </c>
@@ -4543,19 +5324,22 @@
         <v>143</v>
       </c>
       <c r="C16" s="1" t="s">
+        <v>706</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="E16" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>148</v>
       </c>
@@ -4563,19 +5347,22 @@
         <v>149</v>
       </c>
       <c r="C17" s="1" t="s">
+        <v>707</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="E17" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="F17" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="1" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="22" t="s">
         <v>154</v>
       </c>
@@ -4583,19 +5370,22 @@
         <v>94</v>
       </c>
       <c r="C18" s="9" t="s">
+        <v>699</v>
+      </c>
+      <c r="D18" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="E18" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="E18" s="9" t="s">
+      <c r="F18" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="F18" s="9" t="s">
+      <c r="G18" s="9" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="153" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" ht="153" x14ac:dyDescent="0.2">
       <c r="A19" s="22" t="s">
         <v>155</v>
       </c>
@@ -4603,19 +5393,22 @@
         <v>633</v>
       </c>
       <c r="C19" s="18" t="s">
+        <v>708</v>
+      </c>
+      <c r="D19" s="18" t="s">
         <v>634</v>
       </c>
-      <c r="D19" s="18" t="s">
+      <c r="E19" s="18" t="s">
         <v>635</v>
       </c>
-      <c r="E19" s="18" t="s">
+      <c r="F19" s="18" t="s">
         <v>636</v>
       </c>
-      <c r="F19" s="18" t="s">
+      <c r="G19" s="18" t="s">
         <v>637</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="22" t="s">
         <v>156</v>
       </c>
@@ -4623,19 +5416,22 @@
         <v>157</v>
       </c>
       <c r="C20" s="9" t="s">
+        <v>654</v>
+      </c>
+      <c r="D20" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="E20" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="E20" s="9" t="s">
+      <c r="F20" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="G20" s="9" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="22" t="s">
         <v>162</v>
       </c>
@@ -4643,19 +5439,22 @@
         <v>163</v>
       </c>
       <c r="C21" s="9" t="s">
+        <v>655</v>
+      </c>
+      <c r="D21" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="E21" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="E21" s="9" t="s">
+      <c r="F21" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="F21" s="9" t="s">
+      <c r="G21" s="9" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" s="22" t="s">
         <v>168</v>
       </c>
@@ -4663,19 +5462,22 @@
         <v>41</v>
       </c>
       <c r="C22" s="9" t="s">
+        <v>645</v>
+      </c>
+      <c r="D22" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="E22" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="E22" s="9" t="s">
+      <c r="F22" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="F22" s="9" t="s">
+      <c r="G22" s="9" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="22" t="s">
         <v>169</v>
       </c>
@@ -4683,19 +5485,22 @@
         <v>170</v>
       </c>
       <c r="C23" s="9" t="s">
+        <v>709</v>
+      </c>
+      <c r="D23" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="D23" s="9" t="s">
+      <c r="E23" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="E23" s="9" t="s">
+      <c r="F23" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="F23" s="9" t="s">
+      <c r="G23" s="9" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="22" t="s">
         <v>175</v>
       </c>
@@ -4703,19 +5508,22 @@
         <v>176</v>
       </c>
       <c r="C24" s="9" t="s">
+        <v>710</v>
+      </c>
+      <c r="D24" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="D24" s="9" t="s">
+      <c r="E24" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="E24" s="9" t="s">
+      <c r="F24" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="F24" s="9" t="s">
+      <c r="G24" s="9" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" s="22" t="s">
         <v>181</v>
       </c>
@@ -4723,19 +5531,22 @@
         <v>88</v>
       </c>
       <c r="C25" s="9" t="s">
+        <v>698</v>
+      </c>
+      <c r="D25" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="E25" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="E25" s="9" t="s">
+      <c r="F25" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="F25" s="9" t="s">
+      <c r="G25" s="9" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="22" t="s">
         <v>182</v>
       </c>
@@ -4743,19 +5554,22 @@
         <v>183</v>
       </c>
       <c r="C26" s="9" t="s">
+        <v>711</v>
+      </c>
+      <c r="D26" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="E26" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="E26" s="9" t="s">
+      <c r="F26" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="F26" s="9" t="s">
+      <c r="G26" s="9" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" s="22" t="s">
         <v>188</v>
       </c>
@@ -4763,19 +5577,22 @@
         <v>189</v>
       </c>
       <c r="C27" s="9" t="s">
+        <v>712</v>
+      </c>
+      <c r="D27" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="E27" s="9" t="s">
         <v>191</v>
       </c>
-      <c r="E27" s="9" t="s">
+      <c r="F27" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="F27" s="9" t="s">
+      <c r="G27" s="9" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" s="22" t="s">
         <v>194</v>
       </c>
@@ -4783,19 +5600,22 @@
         <v>195</v>
       </c>
       <c r="C28" s="9" t="s">
+        <v>713</v>
+      </c>
+      <c r="D28" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="D28" s="9" t="s">
+      <c r="E28" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="E28" s="9" t="s">
+      <c r="F28" s="9" t="s">
         <v>198</v>
       </c>
-      <c r="F28" s="9" t="s">
+      <c r="G28" s="9" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" s="22" t="s">
         <v>200</v>
       </c>
@@ -4803,19 +5623,22 @@
         <v>201</v>
       </c>
       <c r="C29" s="9" t="s">
+        <v>714</v>
+      </c>
+      <c r="D29" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="D29" s="9" t="s">
+      <c r="E29" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="E29" s="9" t="s">
+      <c r="F29" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="F29" s="9" t="s">
+      <c r="G29" s="9" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" s="22" t="s">
         <v>206</v>
       </c>
@@ -4823,19 +5646,22 @@
         <v>207</v>
       </c>
       <c r="C30" s="9" t="s">
+        <v>712</v>
+      </c>
+      <c r="D30" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="D30" s="9" t="s">
+      <c r="E30" s="9" t="s">
         <v>191</v>
       </c>
-      <c r="E30" s="9" t="s">
+      <c r="F30" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="F30" s="9" t="s">
+      <c r="G30" s="9" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" s="22" t="s">
         <v>208</v>
       </c>
@@ -4843,19 +5669,22 @@
         <v>209</v>
       </c>
       <c r="C31" s="9" t="s">
+        <v>713</v>
+      </c>
+      <c r="D31" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="D31" s="9" t="s">
+      <c r="E31" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="E31" s="9" t="s">
+      <c r="F31" s="9" t="s">
         <v>198</v>
       </c>
-      <c r="F31" s="9" t="s">
+      <c r="G31" s="9" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" s="22" t="s">
         <v>210</v>
       </c>
@@ -4863,19 +5692,22 @@
         <v>211</v>
       </c>
       <c r="C32" s="9" t="s">
+        <v>714</v>
+      </c>
+      <c r="D32" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="D32" s="9" t="s">
+      <c r="E32" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="E32" s="9" t="s">
+      <c r="F32" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="F32" s="9" t="s">
+      <c r="G32" s="9" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" s="22" t="s">
         <v>212</v>
       </c>
@@ -4883,19 +5715,22 @@
         <v>170</v>
       </c>
       <c r="C33" s="9" t="s">
+        <v>709</v>
+      </c>
+      <c r="D33" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="D33" s="9" t="s">
+      <c r="E33" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="E33" s="9" t="s">
+      <c r="F33" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="F33" s="9" t="s">
+      <c r="G33" s="9" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" s="22" t="s">
         <v>213</v>
       </c>
@@ -4903,29 +5738,33 @@
         <v>176</v>
       </c>
       <c r="C34" s="9" t="s">
+        <v>710</v>
+      </c>
+      <c r="D34" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="D34" s="9" t="s">
+      <c r="E34" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="E34" s="9" t="s">
+      <c r="F34" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="F34" s="9" t="s">
+      <c r="G34" s="9" t="s">
         <v>180</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58460040-3E2D-46D4-83B3-4D7C67DE9698}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="13.33203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -4933,19 +5772,22 @@
         <v>1</v>
       </c>
       <c r="C1" s="8" t="s">
+        <v>639</v>
+      </c>
+      <c r="D1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="E1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="F1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="G1" s="8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="22" t="s">
         <v>214</v>
       </c>
@@ -4953,19 +5795,22 @@
         <v>215</v>
       </c>
       <c r="C2" s="9" t="s">
+        <v>715</v>
+      </c>
+      <c r="D2" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="E2" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="F2" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="G2" s="9" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="22" t="s">
         <v>220</v>
       </c>
@@ -4973,15 +5818,18 @@
         <v>221</v>
       </c>
       <c r="C3" s="9" t="s">
+        <v>716</v>
+      </c>
+      <c r="D3" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="E3" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="F3" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="G3" s="9" t="s">
         <v>225</v>
       </c>
     </row>
@@ -4992,18 +5840,19 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{189F51C3-7FE3-4CE8-924B-C200BFCBF56D}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="19.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="58.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="53.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="40" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="44.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="58.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="53.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="44.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -5011,19 +5860,22 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>639</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>255</v>
       </c>
@@ -5031,19 +5883,22 @@
         <v>256</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>717</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>261</v>
       </c>
@@ -5051,19 +5906,22 @@
         <v>262</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>718</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>267</v>
       </c>
@@ -5071,19 +5929,22 @@
         <v>268</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>721</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>357</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="F4" s="19" t="s">
         <v>269</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>271</v>
       </c>
@@ -5091,19 +5952,22 @@
         <v>272</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>277</v>
       </c>
@@ -5111,19 +5975,22 @@
         <v>278</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>720</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>283</v>
       </c>
@@ -5131,15 +5998,18 @@
         <v>284</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>722</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>288</v>
       </c>
     </row>
@@ -5151,18 +6021,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28D3608B-1AB4-CF4B-BF63-C6B6798FA1B2}">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="35.1640625" customWidth="1"/>
+    <col min="3" max="3" width="34.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="41.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="39.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="35.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -5170,19 +6041,22 @@
         <v>1</v>
       </c>
       <c r="C1" s="10" t="s">
+        <v>639</v>
+      </c>
+      <c r="D1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="E1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="F1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="G1" s="10" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="14" t="s">
         <v>350</v>
       </c>
@@ -5190,19 +6064,22 @@
         <v>351</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>723</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="14" t="s">
         <v>356</v>
       </c>
@@ -5210,19 +6087,22 @@
         <v>268</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>721</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>357</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="14" t="s">
         <v>359</v>
       </c>
@@ -5230,19 +6110,22 @@
         <v>360</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>724</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>361</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>362</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="14" t="s">
         <v>365</v>
       </c>
@@ -5250,19 +6133,22 @@
         <v>366</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>367</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>368</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>369</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>370</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
         <v>371</v>
       </c>
@@ -5270,19 +6156,22 @@
         <v>372</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>726</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>373</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>374</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>375</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="14" t="s">
         <v>377</v>
       </c>
@@ -5290,19 +6179,22 @@
         <v>378</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>732</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>379</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>381</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>289</v>
       </c>
@@ -5310,19 +6202,22 @@
         <v>290</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>728</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>295</v>
       </c>
@@ -5330,19 +6225,22 @@
         <v>290</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>728</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>296</v>
       </c>
@@ -5350,19 +6248,22 @@
         <v>297</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>729</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>299</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>302</v>
       </c>
@@ -5370,19 +6271,22 @@
         <v>176</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>710</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="E11" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="F11" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>303</v>
       </c>
@@ -5390,19 +6294,22 @@
         <v>304</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>730</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="D12" s="20" t="s">
+      <c r="E12" s="20" t="s">
         <v>306</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>307</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>309</v>
       </c>
@@ -5410,19 +6317,22 @@
         <v>310</v>
       </c>
       <c r="C13" s="1" t="s">
+        <v>731</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>536</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="E13" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="22" t="s">
         <v>314</v>
       </c>
@@ -5430,19 +6340,22 @@
         <v>315</v>
       </c>
       <c r="C14" s="9" t="s">
+        <v>733</v>
+      </c>
+      <c r="D14" s="9" t="s">
         <v>316</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="E14" s="9" t="s">
         <v>317</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="F14" s="9" t="s">
         <v>318</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="G14" s="9" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="22" t="s">
         <v>320</v>
       </c>
@@ -5450,19 +6363,22 @@
         <v>321</v>
       </c>
       <c r="C15" s="11" t="s">
+        <v>734</v>
+      </c>
+      <c r="D15" s="11" t="s">
         <v>322</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="E15" s="11" t="s">
         <v>323</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="F15" s="11" t="s">
         <v>324</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="G15" s="11" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="22" t="s">
         <v>326</v>
       </c>
@@ -5470,19 +6386,22 @@
         <v>327</v>
       </c>
       <c r="C16" s="9" t="s">
+        <v>735</v>
+      </c>
+      <c r="D16" s="9" t="s">
         <v>328</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="E16" s="9" t="s">
         <v>329</v>
       </c>
-      <c r="E16" s="9" t="s">
+      <c r="F16" s="9" t="s">
         <v>330</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="G16" s="9" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="22" t="s">
         <v>332</v>
       </c>
@@ -5490,19 +6409,22 @@
         <v>333</v>
       </c>
       <c r="C17" s="9" t="s">
+        <v>736</v>
+      </c>
+      <c r="D17" s="9" t="s">
         <v>334</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="E17" s="9" t="s">
         <v>335</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="F17" s="9" t="s">
         <v>336</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="G17" s="9" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="22" t="s">
         <v>338</v>
       </c>
@@ -5510,19 +6432,22 @@
         <v>339</v>
       </c>
       <c r="C18" s="9" t="s">
+        <v>737</v>
+      </c>
+      <c r="D18" s="9" t="s">
         <v>340</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="E18" s="9" t="s">
         <v>341</v>
       </c>
-      <c r="E18" s="9" t="s">
+      <c r="F18" s="9" t="s">
         <v>342</v>
       </c>
-      <c r="F18" s="9" t="s">
+      <c r="G18" s="9" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="22" t="s">
         <v>344</v>
       </c>
@@ -5530,35 +6455,39 @@
         <v>345</v>
       </c>
       <c r="C19" s="11" t="s">
+        <v>738</v>
+      </c>
+      <c r="D19" s="11" t="s">
         <v>346</v>
       </c>
-      <c r="D19" s="11" t="s">
+      <c r="E19" s="11" t="s">
         <v>347</v>
       </c>
-      <c r="E19" s="11" t="s">
+      <c r="F19" s="11" t="s">
         <v>348</v>
       </c>
-      <c r="F19" s="11" t="s">
+      <c r="G19" s="11" t="s">
         <v>349</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1E11308-35D0-4E1E-8C0B-5C10455A0919}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="26.1640625" customWidth="1"/>
-    <col min="3" max="3" width="30.1640625" customWidth="1"/>
-    <col min="4" max="4" width="32.6640625" customWidth="1"/>
-    <col min="5" max="6" width="26.1640625" customWidth="1"/>
+    <col min="1" max="3" width="26.1640625" customWidth="1"/>
+    <col min="4" max="4" width="30.1640625" customWidth="1"/>
+    <col min="5" max="5" width="32.6640625" customWidth="1"/>
+    <col min="6" max="7" width="26.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -5566,19 +6495,22 @@
         <v>1</v>
       </c>
       <c r="C1" s="17" t="s">
+        <v>639</v>
+      </c>
+      <c r="D1" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="E1" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="F1" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="G1" s="17" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>537</v>
       </c>
@@ -5586,39 +6518,45 @@
         <v>538</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>763</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>539</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>542</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>543</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>417</v>
+        <v>768</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>418</v>
+        <v>764</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>419</v>
+        <v>769</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>420</v>
+        <v>770</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+        <v>771</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>544</v>
       </c>
@@ -5626,19 +6564,22 @@
         <v>545</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>765</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>546</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>547</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>548</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>549</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>550</v>
       </c>
@@ -5646,19 +6587,22 @@
         <v>560</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>766</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>558</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>556</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>552</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>551</v>
       </c>
@@ -5666,19 +6610,22 @@
         <v>561</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>767</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>559</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>555</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>562</v>
       </c>
@@ -5686,19 +6633,22 @@
         <v>390</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>755</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>563</v>
       </c>
@@ -5706,19 +6656,22 @@
         <v>423</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>760</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>424</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>425</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>426</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>564</v>
       </c>
@@ -5726,19 +6679,22 @@
         <v>429</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>761</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>431</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>432</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>433</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>565</v>
       </c>
@@ -5746,19 +6702,22 @@
         <v>170</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>709</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>566</v>
       </c>
@@ -5766,15 +6725,18 @@
         <v>176</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>710</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="E11" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="F11" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>180</v>
       </c>
     </row>

</xml_diff>